<commit_message>
Recalibrate pricing tables with 2026 Portuguese market rates and document sources
Co-authored-by: edu18082001 <edu18082001@gmail.com>
</commit_message>
<xml_diff>
--- a/Calculadora_Precos_esDEV.xlsx
+++ b/Calculadora_Precos_esDEV.xlsx
@@ -931,11 +931,11 @@
     <row r="32" ht="30" customHeight="1">
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Plano Essencial</t>
+          <t>Plano Basic</t>
         </is>
       </c>
       <c r="C32" s="19">
-        <f>MAX(Parametros!$C$66,ROUND($C$27*Parametros!$B$66,0))</f>
+        <f>MIN(Parametros!$D$66,MAX(Parametros!$C$66,ROUND($C$27*Parametros!$B$66,0)))</f>
         <v/>
       </c>
       <c r="D32" s="20">
@@ -944,18 +944,18 @@
       </c>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t>Alojamento, updates de segurança, backups, 1h/mês de alterações, resposta em 3 dias úteis.</t>
+          <t>Alojamento, atualizações de segurança, SSL, backups testados, monitorização e pequenas correções.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Plano Pro</t>
+          <t>Plano Business</t>
         </is>
       </c>
       <c r="C33" s="19">
-        <f>MAX(Parametros!$C$67,ROUND($C$27*Parametros!$B$67,0))</f>
+        <f>MIN(Parametros!$D$67,MAX(Parametros!$C$67,ROUND($C$27*Parametros!$B$67,0)))</f>
         <v/>
       </c>
       <c r="D33" s="20">
@@ -964,18 +964,18 @@
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t>Tudo do Essencial + monitorização, 3h/mês de alterações, relatório trimestral, resposta em 1 dia útil.</t>
+          <t>Basic + 2h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Plano Premium</t>
+          <t>Plano Pro</t>
         </is>
       </c>
       <c r="C34" s="19">
-        <f>MAX(Parametros!$C$68,ROUND($C$27*Parametros!$B$68,0))</f>
+        <f>MIN(Parametros!$D$68,MAX(Parametros!$C$68,ROUND($C$27*Parametros!$B$68,0)))</f>
         <v/>
       </c>
       <c r="D34" s="20">
@@ -984,7 +984,7 @@
       </c>
       <c r="E34" s="17" t="inlineStr">
         <is>
-          <t>Tudo do Pro + 6h/mês de evolução, prioridade absoluta, SLA 4h úteis, reunião mensal.</t>
+          <t>Business + 5h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -1532,7 +1532,7 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7">
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="B10" s="39" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="B11" s="39" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="B12" s="39" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -1758,28 +1758,28 @@
         </is>
       </c>
       <c r="B27" s="44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="44" t="n">
         <v>6</v>
-      </c>
-      <c r="D27" s="44" t="n">
-        <v>14</v>
       </c>
       <c r="E27" s="44" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" s="44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H27" s="44" t="n">
         <v>1</v>
       </c>
       <c r="I27" s="45" t="n">
-        <v>450</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28">
@@ -1789,28 +1789,28 @@
         </is>
       </c>
       <c r="B28" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="44" t="n">
+        <v>16</v>
+      </c>
+      <c r="E28" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="44" t="n">
         <v>4</v>
-      </c>
-      <c r="C28" s="44" t="n">
-        <v>12</v>
-      </c>
-      <c r="D28" s="44" t="n">
-        <v>28</v>
-      </c>
-      <c r="E28" s="44" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" s="44" t="n">
-        <v>4</v>
-      </c>
-      <c r="G28" s="44" t="n">
-        <v>6</v>
       </c>
       <c r="H28" s="44" t="n">
         <v>5</v>
       </c>
       <c r="I28" s="45" t="n">
-        <v>950</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="29">
@@ -1820,28 +1820,28 @@
         </is>
       </c>
       <c r="B29" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="44" t="n">
+        <v>22</v>
+      </c>
+      <c r="E29" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="44" t="n">
         <v>6</v>
-      </c>
-      <c r="C29" s="44" t="n">
-        <v>16</v>
-      </c>
-      <c r="D29" s="44" t="n">
-        <v>40</v>
-      </c>
-      <c r="E29" s="44" t="n">
-        <v>16</v>
-      </c>
-      <c r="F29" s="44" t="n">
-        <v>6</v>
-      </c>
-      <c r="G29" s="44" t="n">
-        <v>10</v>
       </c>
       <c r="H29" s="44" t="n">
         <v>8</v>
       </c>
       <c r="I29" s="45" t="n">
-        <v>1500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="30">
@@ -1851,28 +1851,28 @@
         </is>
       </c>
       <c r="B30" s="44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="44" t="n">
+        <v>14</v>
+      </c>
+      <c r="D30" s="44" t="n">
+        <v>36</v>
+      </c>
+      <c r="E30" s="44" t="n">
+        <v>22</v>
+      </c>
+      <c r="F30" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="C30" s="44" t="n">
-        <v>24</v>
-      </c>
-      <c r="D30" s="44" t="n">
-        <v>70</v>
-      </c>
-      <c r="E30" s="44" t="n">
-        <v>40</v>
-      </c>
-      <c r="F30" s="44" t="n">
-        <v>20</v>
-      </c>
       <c r="G30" s="44" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H30" s="44" t="n">
         <v>10</v>
       </c>
       <c r="I30" s="45" t="n">
-        <v>2900</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="31">
@@ -1882,28 +1882,28 @@
         </is>
       </c>
       <c r="B31" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" s="44" t="n">
+        <v>16</v>
+      </c>
+      <c r="D31" s="44" t="n">
+        <v>50</v>
+      </c>
+      <c r="E31" s="44" t="n">
+        <v>55</v>
+      </c>
+      <c r="F31" s="44" t="n">
         <v>14</v>
       </c>
-      <c r="C31" s="44" t="n">
-        <v>24</v>
-      </c>
-      <c r="D31" s="44" t="n">
-        <v>90</v>
-      </c>
-      <c r="E31" s="44" t="n">
-        <v>90</v>
-      </c>
-      <c r="F31" s="44" t="n">
-        <v>24</v>
-      </c>
       <c r="G31" s="44" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H31" s="44" t="n">
         <v>8</v>
       </c>
       <c r="I31" s="45" t="n">
-        <v>4500</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="32">
@@ -1913,28 +1913,28 @@
         </is>
       </c>
       <c r="B32" s="44" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C32" s="44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" s="44" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E32" s="44" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="F32" s="44" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="G32" s="44" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H32" s="44" t="n">
         <v>1</v>
       </c>
       <c r="I32" s="45" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="33">
@@ -1944,28 +1944,28 @@
         </is>
       </c>
       <c r="B33" s="44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33" s="44" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D33" s="44" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="E33" s="44" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F33" s="44" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G33" s="44" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H33" s="44" t="n">
         <v>5</v>
       </c>
       <c r="I33" s="45" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -2238,6 +2238,11 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
+          <t>Máximo / mês</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
           <t>Inclui</t>
         </is>
       </c>
@@ -2245,54 +2250,63 @@
     <row r="66">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t>Essencial</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="B66" s="47" t="n">
         <v>0.02</v>
       </c>
       <c r="C66" s="45" t="n">
-        <v>39</v>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Alojamento, updates de segurança, backups, 1h/mês de alterações, resposta em 3 dias úteis.</t>
+        <v>45</v>
+      </c>
+      <c r="D66" s="45" t="n">
+        <v>95</v>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Alojamento, atualizações de segurança, SSL, backups testados, monitorização e pequenas correções.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="37" t="inlineStr">
         <is>
-          <t>Pro</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="B67" s="47" t="n">
         <v>0.035</v>
       </c>
       <c r="C67" s="45" t="n">
-        <v>89</v>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>Tudo do Essencial + monitorização, 3h/mês de alterações, relatório trimestral, resposta em 1 dia útil.</t>
+        <v>130</v>
+      </c>
+      <c r="D67" s="45" t="n">
+        <v>280</v>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Basic + 2h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="37" t="inlineStr">
         <is>
-          <t>Premium</t>
+          <t>Pro</t>
         </is>
       </c>
       <c r="B68" s="47" t="n">
         <v>0.055</v>
       </c>
       <c r="C68" s="45" t="n">
-        <v>149</v>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Tudo do Pro + 6h/mês de evolução, prioridade absoluta, SLA 4h úteis, reunião mensal.</t>
+        <v>320</v>
+      </c>
+      <c r="D68" s="45" t="n">
+        <v>650</v>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Business + 5h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2466,7 @@
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Manutenção mensal recomendada (Pro)</t>
+          <t>Manutenção mensal recomendada (Business)</t>
         </is>
       </c>
       <c r="C16" s="48">

</xml_diff>

<commit_message>
Recalibrate prices for a solo freelancer and split the hourly rate into floor and target
Co-authored-by: edu18082001 <edu18082001@gmail.com>
</commit_message>
<xml_diff>
--- a/Calculadora_Precos_esDEV.xlsx
+++ b/Calculadora_Precos_esDEV.xlsx
@@ -964,7 +964,7 @@
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t>Basic + 2h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
+          <t>Basic + 1,5h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="E34" s="17" t="inlineStr">
         <is>
-          <t>Business + 5h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
+          <t>Business + 4h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="B4" s="39" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="B5" s="39" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
@@ -1532,7 +1532,7 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="B7" s="39" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="B8" s="39" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="B10" s="39" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11">
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="B11" s="39" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12">
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="B12" s="39" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -1779,7 +1779,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="45" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
     </row>
     <row r="28">
@@ -1810,7 +1810,7 @@
         <v>5</v>
       </c>
       <c r="I28" s="45" t="n">
-        <v>1900</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="29">
@@ -1841,7 +1841,7 @@
         <v>8</v>
       </c>
       <c r="I29" s="45" t="n">
-        <v>3000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="30">
@@ -1872,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="I30" s="45" t="n">
-        <v>2400</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="31">
@@ -1903,7 +1903,7 @@
         <v>8</v>
       </c>
       <c r="I31" s="45" t="n">
-        <v>9000</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="32">
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="45" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="33">
@@ -1965,7 +1965,7 @@
         <v>5</v>
       </c>
       <c r="I33" s="45" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
@@ -2257,10 +2257,10 @@
         <v>0.02</v>
       </c>
       <c r="C66" s="45" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D66" s="45" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
@@ -2278,14 +2278,14 @@
         <v>0.035</v>
       </c>
       <c r="C67" s="45" t="n">
-        <v>130</v>
+        <v>99</v>
       </c>
       <c r="D67" s="45" t="n">
-        <v>280</v>
+        <v>199</v>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Basic + 2h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
+          <t>Basic + 1,5h/mês de alterações de conteúdo, suporte prioritário em 1 dia útil, relatório trimestral.</t>
         </is>
       </c>
     </row>
@@ -2299,14 +2299,14 @@
         <v>0.055</v>
       </c>
       <c r="C68" s="45" t="n">
-        <v>320</v>
+        <v>249</v>
       </c>
       <c r="D68" s="45" t="n">
-        <v>650</v>
+        <v>450</v>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Business + 5h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
+          <t>Business + 4h/mês de evolução, SEO contínuo, relatório mensal, SLA de 4h úteis e reunião mensal.</t>
         </is>
       </c>
     </row>

</xml_diff>